<commit_message>
feat: enrich tutorial relational scenarios
</commit_message>
<xml_diff>
--- a/data/source/material_workbench_tutorial_v1.xlsx
+++ b/data/source/material_workbench_tutorial_v1.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概要" sheetId="1" r:id="Rf8efd008c51946ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="relation" sheetId="2" r:id="Re9554ff833e14a9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="溶製" sheetId="3" r:id="Rc58bcba3a0f44622"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="熱延" sheetId="4" r:id="Rd4cc65c2b5464579"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="冷延" sheetId="5" r:id="R131d6c61e0fb430e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="焼鈍" sheetId="6" r:id="Rcdff7aa2bcf54f89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="焼鈍履歴" sheetId="7" r:id="Rfbddb3a4fabb43a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="熱延引張" sheetId="8" r:id="R9b1a90a3ff524c3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="熱延組織" sheetId="9" r:id="Rd32947d7f0364d82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="焼鈍引張" sheetId="10" r:id="R6372b0a6c7104718"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="焼鈍穴広げ" sheetId="11" r:id="Rf9e74c352d944cdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="焼鈍組織" sheetId="12" r:id="Ra4600eb6341f42f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="想定異常" sheetId="13" r:id="Re4a92fd3cc8446e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="焼鈍特徴量" sheetId="14" r:id="R23986d9d536848e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概要" sheetId="1" r:id="R731d01922d7046b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="relation" sheetId="2" r:id="Rb6325408086f4eeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="溶製" sheetId="3" r:id="R818dab9e091c4646"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="熱延" sheetId="4" r:id="Rf3de0fe6168d499d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="冷延" sheetId="5" r:id="R9e4358e895a54bbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="焼鈍" sheetId="6" r:id="R76cb6e1290b64995"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="焼鈍履歴" sheetId="7" r:id="R7e65081d018d4974"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="熱延引張" sheetId="8" r:id="R5a56ff2e30674cbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="熱延組織" sheetId="9" r:id="R865ebfb0e4a34b52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="焼鈍引張" sheetId="10" r:id="Rc3916b9488634f2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="焼鈍穴広げ" sheetId="11" r:id="Rfeedd9cd236c4898"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="焼鈍組織" sheetId="12" r:id="R994434fd420f48c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="想定異常" sheetId="13" r:id="R7526397b70eb429d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="焼鈍特徴量" sheetId="14" r:id="R3b7f59beef85480b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -292,68 +292,68 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>成分ロット</x:v>
-      </x:c>
-      <x:c r="B3" t="n">
-        <x:v>4</x:v>
+        <x:v>規模</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>4成分・6熱延・6焼鈍</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>C×Mnの2水準。その他の元素は固定</x:v>
+        <x:v>キーを覚えられる規模は維持する</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>熱延条件</x:v>
-      </x:c>
-      <x:c r="B4" t="n">
-        <x:v>6</x:v>
+        <x:v>共有工程</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>2成分</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>同じ成分で仕上温度だけ違う対を含む</x:v>
+        <x:v>ME-01とME-02がHR-02／CR-02／AN-02を共有する</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>焼鈍条件</x:v>
-      </x:c>
-      <x:c r="B5" t="n">
-        <x:v>6</x:v>
+        <x:v>LSなし焼鈍</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>1条件</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>LSと最高温度の違いを追える</x:v>
+        <x:v>AN-06はLSなし。明示した実測ヒートパターンを正本にする</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>試験</x:v>
+        <x:v>反復</x:v>
       </x:c>
       <x:c r="B6" t="n">
-        <x:v>26</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>熱延引張8・焼鈍引張10・穴広げ8</x:v>
+        <x:v>同じ成分×工程コンテキストへ別の試験IDを結ぶ</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>反復</x:v>
+        <x:v>部分欠損</x:v>
       </x:c>
       <x:c r="B7" t="n">
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>同じ工程条件へ別の試験IDを結ぶ</x:v>
+        <x:v>有効試験の一部目的変数だけを意図的に空欄にする</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>部分欠損</x:v>
-      </x:c>
-      <x:c r="B8" t="n">
-        <x:v>2</x:v>
+        <x:v>分割relation</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>1経路</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>反復行のYS/ELに意図的な空欄</x:v>
+        <x:v>HT-01→HR-01とHR-01→ME-01を別行にして一意に辿る</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -364,7 +364,7 @@
         <x:v>relation</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>relationはリンク。試験行を学習観測として扱う</x:v>
+        <x:v>relation行は経路。工程キーだけで成分を逆引きしない</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -533,11 +533,11 @@
         <x:v>TT-03</x:v>
       </x:c>
       <x:c r="B4" t="n">
-        <x:v>512</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="C4"/>
       <x:c r="D4" t="n">
-        <x:v>28</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E4" t="n">
         <x:v>24</x:v>
@@ -566,7 +566,9 @@
       <x:c r="O4" t="str">
         <x:v>demo</x:v>
       </x:c>
-      <x:c r="P4"/>
+      <x:c r="P4" t="str">
+        <x:v>AN-02をME-01と共有するME-02。YSのみ欠損</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
@@ -992,7 +994,7 @@
         <x:v>HE-03</x:v>
       </x:c>
       <x:c r="B4" t="n">
-        <x:v>104</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="C4" t="n">
         <x:v>10</x:v>
@@ -1019,7 +1021,9 @@
       <x:c r="K4" t="str">
         <x:v>demo</x:v>
       </x:c>
-      <x:c r="L4"/>
+      <x:c r="L4" t="str">
+        <x:v>AN-02をME-01と共有するME-02の試験</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
@@ -1563,9 +1567,7 @@
       <x:c r="E7" t="str">
         <x:v>SOAK</x:v>
       </x:c>
-      <x:c r="F7" t="n">
-        <x:v>60</x:v>
-      </x:c>
+      <x:c r="F7"/>
       <x:c r="G7" t="n">
         <x:v>20</x:v>
       </x:c>
@@ -1642,9 +1644,7 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:v>ME-01</x:v>
-      </x:c>
+      <x:c r="A2"/>
       <x:c r="B2" t="str">
         <x:v>HR-01</x:v>
       </x:c>
@@ -1658,7 +1658,7 @@
       <x:c r="H2"/>
       <x:c r="I2"/>
       <x:c r="J2" t="str">
-        <x:v>熱延引張</x:v>
+        <x:v>分割relation：試験→工程</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1678,12 +1678,12 @@
       <x:c r="H3"/>
       <x:c r="I3"/>
       <x:c r="J3" t="str">
-        <x:v>熱延引張</x:v>
+        <x:v>共有工程：成分A</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>ME-01</x:v>
+        <x:v>ME-02</x:v>
       </x:c>
       <x:c r="B4" t="str">
         <x:v>HR-02</x:v>
@@ -1698,7 +1698,7 @@
       <x:c r="H4"/>
       <x:c r="I4"/>
       <x:c r="J4" t="str">
-        <x:v>熱延引張</x:v>
+        <x:v>共有工程：成分B</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1846,12 +1846,12 @@
       <x:c r="H11"/>
       <x:c r="I11"/>
       <x:c r="J11" t="str">
-        <x:v>焼鈍引張</x:v>
+        <x:v>共有焼鈍：成分A</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>ME-01</x:v>
+        <x:v>ME-02</x:v>
       </x:c>
       <x:c r="B12" t="str">
         <x:v>HR-02</x:v>
@@ -1870,7 +1870,7 @@
       <x:c r="H12"/>
       <x:c r="I12"/>
       <x:c r="J12" t="str">
-        <x:v>焼鈍引張</x:v>
+        <x:v>共有焼鈍：成分B</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2086,12 +2086,12 @@
       </x:c>
       <x:c r="I21"/>
       <x:c r="J21" t="str">
-        <x:v>焼鈍穴広げ</x:v>
+        <x:v>共有焼鈍：成分A</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
-        <x:v>ME-01</x:v>
+        <x:v>ME-02</x:v>
       </x:c>
       <x:c r="B22" t="str">
         <x:v>HR-02</x:v>
@@ -2110,7 +2110,7 @@
       </x:c>
       <x:c r="I22"/>
       <x:c r="J22" t="str">
-        <x:v>焼鈍穴広げ</x:v>
+        <x:v>共有焼鈍：成分B</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -2231,6 +2231,24 @@
       <x:c r="I27"/>
       <x:c r="J27" t="str">
         <x:v>焼鈍穴広げ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>ME-01</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>HR-01</x:v>
+      </x:c>
+      <x:c r="C28"/>
+      <x:c r="D28"/>
+      <x:c r="E28"/>
+      <x:c r="F28"/>
+      <x:c r="G28"/>
+      <x:c r="H28"/>
+      <x:c r="I28"/>
+      <x:c r="J28" t="str">
+        <x:v>分割relation：工程→成分</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3672,9 +3690,7 @@
       <x:c r="A7" t="str">
         <x:v>AN-06</x:v>
       </x:c>
-      <x:c r="B7" t="n">
-        <x:v>60</x:v>
-      </x:c>
+      <x:c r="B7"/>
       <x:c r="C7" t="str">
         <x:v>CAL-DEMO</x:v>
       </x:c>
@@ -3727,7 +3743,9 @@
       <x:c r="T7" t="str">
         <x:v>学習</x:v>
       </x:c>
-      <x:c r="U7"/>
+      <x:c r="U7" t="str">
+        <x:v>LSなし。焼鈍履歴の経過時間と実績温度を使用</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5086,11 +5104,9 @@
       <x:c r="I32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J32" t="n">
-        <x:v>60</x:v>
-      </x:c>
+      <x:c r="J32"/>
       <x:c r="K32" t="str">
-        <x:v>教材値</x:v>
+        <x:v>経過時間指定</x:v>
       </x:c>
       <x:c r="L32" t="str">
         <x:v>demo</x:v>
@@ -5098,7 +5114,9 @@
       <x:c r="M32" t="str">
         <x:v>辞書一致</x:v>
       </x:c>
-      <x:c r="N32"/>
+      <x:c r="N32" t="str">
+        <x:v>LSなし・実測履歴を正本</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="str">
@@ -5128,11 +5146,9 @@
       <x:c r="I33" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="J33" t="n">
-        <x:v>60</x:v>
-      </x:c>
+      <x:c r="J33"/>
       <x:c r="K33" t="str">
-        <x:v>教材値</x:v>
+        <x:v>経過時間指定</x:v>
       </x:c>
       <x:c r="L33" t="str">
         <x:v>demo</x:v>
@@ -5170,11 +5186,9 @@
       <x:c r="I34" t="n">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="J34" t="n">
-        <x:v>60</x:v>
-      </x:c>
+      <x:c r="J34"/>
       <x:c r="K34" t="str">
-        <x:v>教材値</x:v>
+        <x:v>経過時間指定</x:v>
       </x:c>
       <x:c r="L34" t="str">
         <x:v>demo</x:v>
@@ -5212,11 +5226,9 @@
       <x:c r="I35" t="n">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="J35" t="n">
-        <x:v>60</x:v>
-      </x:c>
+      <x:c r="J35"/>
       <x:c r="K35" t="str">
-        <x:v>教材値</x:v>
+        <x:v>経過時間指定</x:v>
       </x:c>
       <x:c r="L35" t="str">
         <x:v>demo</x:v>
@@ -5254,11 +5266,9 @@
       <x:c r="I36" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="J36" t="n">
-        <x:v>60</x:v>
-      </x:c>
+      <x:c r="J36"/>
       <x:c r="K36" t="str">
-        <x:v>教材値</x:v>
+        <x:v>経過時間指定</x:v>
       </x:c>
       <x:c r="L36" t="str">
         <x:v>demo</x:v>
@@ -5296,11 +5306,9 @@
       <x:c r="I37" t="n">
         <x:v>240</x:v>
       </x:c>
-      <x:c r="J37" t="n">
-        <x:v>60</x:v>
-      </x:c>
+      <x:c r="J37"/>
       <x:c r="K37" t="str">
-        <x:v>教材値</x:v>
+        <x:v>経過時間指定</x:v>
       </x:c>
       <x:c r="L37" t="str">
         <x:v>demo</x:v>
@@ -5464,12 +5472,14 @@
         <x:v>HT-03</x:v>
       </x:c>
       <x:c r="B4" t="n">
-        <x:v>472</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="C4" t="n">
-        <x:v>316</x:v>
-      </x:c>
-      <x:c r="D4"/>
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="D4" t="n">
+        <x:v>27</x:v>
+      </x:c>
       <x:c r="E4"/>
       <x:c r="F4" t="str">
         <x:v>L</x:v>
@@ -5493,7 +5503,9 @@
       <x:c r="M4" t="str">
         <x:v>demo</x:v>
       </x:c>
-      <x:c r="N4"/>
+      <x:c r="N4" t="str">
+        <x:v>HR-02をME-01と共有するME-02の試験</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">

</xml_diff>